<commit_message>
auto: snapshot 2026-07-15 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -457,7 +457,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-15 13:01:00</t>
+          <t>Timestamp: 2026-07-15 13:31:00</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>13464</v>
+        <v>13489</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>13142</v>
+        <v>13167</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>13179</v>
+        <v>13204</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>13158</v>
+        <v>13183</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>12912</v>
+        <v>12937</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>12998</v>
+        <v>13023</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>12659</v>
+        <v>12684</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>12404</v>
+        <v>12429</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>12609</v>
+        <v>12634</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>10553</v>
+        <v>10578</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>10423</v>
+        <v>10448</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>10076</v>
+        <v>10101</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>9980</v>
+        <v>10005</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>9903</v>
+        <v>9928</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
@@ -1250,7 +1250,7 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>12469</v>
+        <v>12494</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>5444</v>
+        <v>5519</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-22 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -14,6 +14,7 @@
     <sheet name="2026-07-19" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-20" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-21" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-07-22" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6545,4 +6546,868 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-22 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3236</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+682</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3120</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+601</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3189</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>2863</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+663</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>2696</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2705</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>3625</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+665</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3368</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+677</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3158</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+633</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3001</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+576</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2921</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+558</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1238</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+977</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>4743</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+929</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2497</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+697</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4111</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+707</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>3680</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+709</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>3596</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+721</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3382</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+699</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3169</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>The Strategist</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>242</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>4486</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1142</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1653</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1728</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1682</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1706</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+185</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>3734</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1015</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>3854</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+993</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3613</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+913</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3064</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+874</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>456</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>417</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>261</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1326</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1214</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1132</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1706</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1235</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>606</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+381</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>606</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+381</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>670</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+445</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>1036</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>930</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>918</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>887</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>308</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>670</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+445</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>The ArchitectX</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+301</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>355</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+196</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-22 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -6572,7 +6572,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-22 13:01:00</t>
+          <t>Timestamp: 2026-07-22 13:31:00</t>
         </is>
       </c>
     </row>
@@ -6630,11 +6630,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>3120</v>
+        <v>3145</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+601</t>
+          <t>+626</t>
         </is>
       </c>
     </row>
@@ -6645,11 +6645,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3189</v>
+        <v>3214</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
@@ -6660,11 +6660,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>2863</v>
+        <v>2888</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+663</t>
+          <t>+688</t>
         </is>
       </c>
     </row>
@@ -6675,11 +6675,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>2696</v>
+        <v>2721</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -6690,11 +6690,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>2705</v>
+        <v>2730</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+725</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -6705,11 +6705,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>3625</v>
+        <v>3650</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+665</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -6720,11 +6720,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>3368</v>
+        <v>3393</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+677</t>
+          <t>+702</t>
         </is>
       </c>
     </row>
@@ -6735,11 +6735,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>3158</v>
+        <v>3183</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+633</t>
+          <t>+658</t>
         </is>
       </c>
     </row>
@@ -6750,11 +6750,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>3001</v>
+        <v>3026</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+576</t>
+          <t>+601</t>
         </is>
       </c>
     </row>
@@ -6765,11 +6765,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>2921</v>
+        <v>2946</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+558</t>
+          <t>+583</t>
         </is>
       </c>
     </row>
@@ -6795,11 +6795,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>4743</v>
+        <v>4768</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+929</t>
+          <t>+954</t>
         </is>
       </c>
     </row>
@@ -6810,11 +6810,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>2497</v>
+        <v>2522</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+697</t>
+          <t>+722</t>
         </is>
       </c>
     </row>
@@ -6825,11 +6825,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>4111</v>
+        <v>4136</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+707</t>
+          <t>+732</t>
         </is>
       </c>
     </row>
@@ -6840,11 +6840,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>3680</v>
+        <v>3705</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+709</t>
+          <t>+734</t>
         </is>
       </c>
     </row>
@@ -6855,11 +6855,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>3596</v>
+        <v>3621</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+721</t>
+          <t>+746</t>
         </is>
       </c>
     </row>
@@ -6870,11 +6870,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>3382</v>
+        <v>3407</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+699</t>
+          <t>+724</t>
         </is>
       </c>
     </row>
@@ -6885,11 +6885,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3169</v>
+        <v>3194</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+715</t>
         </is>
       </c>
     </row>
@@ -7020,11 +7020,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>3854</v>
+        <v>3934</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+993</t>
+          <t>+1073</t>
         </is>
       </c>
     </row>
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>3613</v>
+        <v>3697</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+913</t>
+          <t>+997</t>
         </is>
       </c>
     </row>
@@ -7050,11 +7050,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3064</v>
+        <v>3139</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+874</t>
+          <t>+949</t>
         </is>
       </c>
     </row>
@@ -7380,11 +7380,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+75</t>
+          <t>+100</t>
         </is>
       </c>
     </row>
@@ -7395,11 +7395,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>355</v>
+        <v>430</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+196</t>
+          <t>+271</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-23 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -15,6 +15,7 @@
     <sheet name="2026-07-20" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-21" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-07-22" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-07-23" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7410,4 +7411,868 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-23 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3932</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+696</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4025</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3889</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3551</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+663</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>3310</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+589</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>3325</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+595</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>4530</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>4243</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4008</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3836</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+810</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>3746</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1238</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+977</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>5614</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+846</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3107</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+585</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4926</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>4531</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+826</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>4396</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+775</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>4152</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+745</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3911</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+717</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>The Strategist</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>367</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5487</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1001</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2241</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+588</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2328</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>2258</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+576</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2296</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+590</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>4657</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+923</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>4922</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+988</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>4697</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>4067</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+928</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>531</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>492</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>336</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1326</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1214</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1132</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2296</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+590</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1235</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1291</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+621</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1217</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+547</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>1198</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+648</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>1256</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+586</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>1036</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>930</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>918</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>887</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>758</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>1244</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+574</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>The ArchitectX</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>530</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-23 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -7437,7 +7437,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-23 13:01:00</t>
+          <t>Timestamp: 2026-07-23 13:31:00</t>
         </is>
       </c>
     </row>
@@ -7495,11 +7495,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4025</v>
+        <v>4050</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -7510,11 +7510,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3889</v>
+        <v>3914</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
@@ -7525,11 +7525,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3551</v>
+        <v>3576</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+663</t>
+          <t>+688</t>
         </is>
       </c>
     </row>
@@ -7540,11 +7540,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>3310</v>
+        <v>3385</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+589</t>
+          <t>+664</t>
         </is>
       </c>
     </row>
@@ -7555,11 +7555,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>3325</v>
+        <v>3400</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+670</t>
         </is>
       </c>
     </row>
@@ -7570,11 +7570,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>4530</v>
+        <v>4555</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -7585,11 +7585,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4243</v>
+        <v>4298</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -7600,11 +7600,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>4008</v>
+        <v>4083</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -7615,11 +7615,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>3836</v>
+        <v>3911</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+885</t>
         </is>
       </c>
     </row>
@@ -7630,11 +7630,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>3746</v>
+        <v>3821</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -7660,11 +7660,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>5614</v>
+        <v>5639</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+846</t>
+          <t>+871</t>
         </is>
       </c>
     </row>
@@ -7675,11 +7675,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>3107</v>
+        <v>3182</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+585</t>
+          <t>+660</t>
         </is>
       </c>
     </row>
@@ -7690,11 +7690,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>4926</v>
+        <v>4951</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+815</t>
         </is>
       </c>
     </row>
@@ -7705,11 +7705,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>4531</v>
+        <v>4556</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+826</t>
+          <t>+851</t>
         </is>
       </c>
     </row>
@@ -7720,11 +7720,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>4396</v>
+        <v>4466</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+775</t>
+          <t>+845</t>
         </is>
       </c>
     </row>
@@ -7735,11 +7735,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>4152</v>
+        <v>4227</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+745</t>
+          <t>+820</t>
         </is>
       </c>
     </row>
@@ -7750,11 +7750,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3911</v>
+        <v>3986</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+717</t>
+          <t>+792</t>
         </is>
       </c>
     </row>
@@ -7795,11 +7795,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2241</v>
+        <v>2266</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+588</t>
+          <t>+613</t>
         </is>
       </c>
     </row>
@@ -7810,11 +7810,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>2328</v>
+        <v>2353</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -7825,11 +7825,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>2258</v>
+        <v>2283</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+576</t>
+          <t>+601</t>
         </is>
       </c>
     </row>
@@ -7840,11 +7840,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2296</v>
+        <v>2321</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+615</t>
         </is>
       </c>
     </row>
@@ -8035,11 +8035,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>2296</v>
+        <v>2321</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+590</t>
+          <t>+615</t>
         </is>
       </c>
     </row>
@@ -8065,11 +8065,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>1291</v>
+        <v>1316</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+621</t>
+          <t>+646</t>
         </is>
       </c>
     </row>
@@ -8080,11 +8080,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>1217</v>
+        <v>1242</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+547</t>
+          <t>+572</t>
         </is>
       </c>
     </row>
@@ -8095,11 +8095,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>1198</v>
+        <v>1238</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+648</t>
+          <t>+688</t>
         </is>
       </c>
     </row>
@@ -8110,11 +8110,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>1256</v>
+        <v>1356</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+586</t>
+          <t>+686</t>
         </is>
       </c>
     </row>
@@ -8215,11 +8215,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>1244</v>
+        <v>1344</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+574</t>
+          <t>+674</t>
         </is>
       </c>
     </row>
@@ -8245,11 +8245,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-25 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -17,6 +17,7 @@
     <sheet name="2026-07-22" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-07-23" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-07-24" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-07-25" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2185,6 +2186,870 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-25 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>5283</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+578</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>5290</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+632</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>5337</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+848</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>4983</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4768</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+848</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>4718</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+803</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>5784</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+643</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>5479</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+615</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>5266</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+623</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>5067</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+596</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>4960</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+579</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1686</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1290</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>7194</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+755</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+783</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>6374</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+823</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>5937</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+797</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>5829</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+745</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>5538</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+707</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>5265</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+687</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>The Strategist</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>402</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7376</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+874</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>4077</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+837</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>4159</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+837</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>4078</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>4051</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+761</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1737</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+364</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6255</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>6732</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+786</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6519</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+802</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>5604</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+624</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>591</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>577</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>396</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1618</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1464</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1337</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>4075</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+763</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1410</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>3022</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+784</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>2921</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+683</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>2947</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+793</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>3212</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+974</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2224</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+744</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2071</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+701</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+666</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>1963</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+691</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>1926</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+699</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>1377</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+319</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>3054</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+816</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>The ArchitectX</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>1121</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>317</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+67</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>830</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -3075,7 +3075,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-26 13:01:00</t>
+          <t>Timestamp: 2026-07-26 13:31:00</t>
         </is>
       </c>
     </row>
@@ -3133,11 +3133,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7040</v>
+        <v>7130</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1700</t>
+          <t>+1790</t>
         </is>
       </c>
     </row>
@@ -3148,11 +3148,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7237</v>
+        <v>7337</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1850</t>
+          <t>+1950</t>
         </is>
       </c>
     </row>
@@ -3163,11 +3163,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6828</v>
+        <v>6928</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+1795</t>
+          <t>+1895</t>
         </is>
       </c>
     </row>
@@ -3178,11 +3178,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>6525</v>
+        <v>6625</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1707</t>
+          <t>+1807</t>
         </is>
       </c>
     </row>
@@ -3193,11 +3193,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>6532</v>
+        <v>6632</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1764</t>
+          <t>+1864</t>
         </is>
       </c>
     </row>
@@ -3208,11 +3208,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>7534</v>
+        <v>7634</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1700</t>
+          <t>+1800</t>
         </is>
       </c>
     </row>
@@ -3223,11 +3223,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7179</v>
+        <v>7279</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1650</t>
+          <t>+1750</t>
         </is>
       </c>
     </row>
@@ -3238,11 +3238,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>6939</v>
+        <v>7039</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1623</t>
+          <t>+1723</t>
         </is>
       </c>
     </row>
@@ -3253,11 +3253,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>6759</v>
+        <v>6859</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1642</t>
+          <t>+1742</t>
         </is>
       </c>
     </row>
@@ -3268,11 +3268,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>6640</v>
+        <v>6740</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1630</t>
+          <t>+1730</t>
         </is>
       </c>
     </row>
@@ -3298,11 +3298,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>9222</v>
+        <v>9272</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1978</t>
+          <t>+2028</t>
         </is>
       </c>
     </row>
@@ -3313,11 +3313,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>6225</v>
+        <v>6325</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1665</t>
+          <t>+1765</t>
         </is>
       </c>
     </row>
@@ -3328,11 +3328,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>8058</v>
+        <v>8208</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1634</t>
+          <t>+1784</t>
         </is>
       </c>
     </row>
@@ -3343,11 +3343,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>7601</v>
+        <v>7751</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1614</t>
+          <t>+1764</t>
         </is>
       </c>
     </row>
@@ -3358,11 +3358,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>7403</v>
+        <v>7553</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1524</t>
+          <t>+1674</t>
         </is>
       </c>
     </row>
@@ -3373,11 +3373,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>7148</v>
+        <v>7298</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1560</t>
+          <t>+1710</t>
         </is>
       </c>
     </row>
@@ -3388,11 +3388,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>6875</v>
+        <v>7025</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1560</t>
+          <t>+1710</t>
         </is>
       </c>
     </row>
@@ -3403,11 +3403,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>9576</v>
+        <v>9726</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2100</t>
+          <t>+2250</t>
         </is>
       </c>
     </row>
@@ -3493,11 +3493,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>8255</v>
+        <v>8405</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1930</t>
+          <t>+2080</t>
         </is>
       </c>
     </row>
@@ -3508,11 +3508,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>8916</v>
+        <v>9066</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2084</t>
+          <t>+2234</t>
         </is>
       </c>
     </row>
@@ -3523,11 +3523,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>8663</v>
+        <v>8813</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2044</t>
+          <t>+2194</t>
         </is>
       </c>
     </row>
@@ -3538,11 +3538,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>7573</v>
+        <v>7723</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1899</t>
+          <t>+2049</t>
         </is>
       </c>
     </row>
@@ -3688,11 +3688,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>4076</v>
+        <v>4176</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+922</t>
+          <t>+1022</t>
         </is>
       </c>
     </row>
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>4041</v>
+        <v>4141</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+887</t>
+          <t>+987</t>
         </is>
       </c>
     </row>
@@ -3718,11 +3718,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>3997</v>
+        <v>4097</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -3733,11 +3733,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>4302</v>
+        <v>4402</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+1148</t>
+          <t>+1248</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>850</v>
+        <v>950</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
@@ -3763,7 +3763,7 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>805</v>
+        <v>905</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
@@ -3868,11 +3868,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>4104</v>
+        <v>4204</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -3883,11 +3883,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>1371</v>
+        <v>1521</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+400</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 13:01:02
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -20,6 +20,7 @@
     <sheet name="2026-07-25" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-07-26" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-07-27" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-07-28" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4810,6 +4811,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-28 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>8598</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+475</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>8641</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+221</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>8912</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>8503</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>8200</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>8161</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>9159</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>8768</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>8554</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>8384</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>8223</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+210</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1686</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1290</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>11372</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7855</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>9668</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+217</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>9246</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>9051</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8823</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8487</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>11801</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+525</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>6185</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+276</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>6384</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>6336</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>6301</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1737</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>10275</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>11141</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+525</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>10879</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+525</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>9566</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>591</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>577</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>396</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1618</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1464</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1337</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>6289</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1410</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>5726</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+122</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>5619</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+15</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>5617</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>6052</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+448</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Minato Namikaze</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>2470</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2425</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2374</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2221</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>2174</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2113</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2076</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>3278</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+551</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>5847</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+243</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>The ArchitectX</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>1521</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>647</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -4835,7 +4835,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:01:00</t>
+          <t>Timestamp: 2026-07-28 13:31:00</t>
         </is>
       </c>
     </row>
@@ -4908,11 +4908,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>8912</v>
+        <v>8937</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -4923,11 +4923,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>8503</v>
+        <v>8528</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -4938,11 +4938,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8200</v>
+        <v>8210</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+285</t>
         </is>
       </c>
     </row>
@@ -5058,11 +5058,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>11372</v>
+        <v>11397</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -5178,11 +5178,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>6185</v>
+        <v>6210</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+276</t>
+          <t>+301</t>
         </is>
       </c>
     </row>
@@ -5193,11 +5193,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>6384</v>
+        <v>6402</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+318</t>
         </is>
       </c>
     </row>
@@ -5208,11 +5208,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>6336</v>
+        <v>6346</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+310</t>
         </is>
       </c>
     </row>
@@ -5508,11 +5508,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>2470</v>
+        <v>2495</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+225</t>
         </is>
       </c>
     </row>
@@ -5523,11 +5523,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>2425</v>
+        <v>2450</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+225</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -5715,7 +5715,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-29 13:01:00</t>
+          <t>Timestamp: 2026-07-29 13:31:00</t>
         </is>
       </c>
     </row>
@@ -5773,11 +5773,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>9547</v>
+        <v>9572</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+906</t>
+          <t>+931</t>
         </is>
       </c>
     </row>
@@ -5848,11 +5848,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>10154</v>
+        <v>10179</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+995</t>
+          <t>+1020</t>
         </is>
       </c>
     </row>
@@ -5863,11 +5863,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>9748</v>
+        <v>9773</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+1005</t>
         </is>
       </c>
     </row>
@@ -5878,11 +5878,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>9522</v>
+        <v>9547</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+968</t>
+          <t>+993</t>
         </is>
       </c>
     </row>
@@ -5893,11 +5893,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>9372</v>
+        <v>9397</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+988</t>
+          <t>+1013</t>
         </is>
       </c>
     </row>
@@ -5908,11 +5908,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>9163</v>
+        <v>9188</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+940</t>
+          <t>+965</t>
         </is>
       </c>
     </row>
@@ -5938,11 +5938,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>12422</v>
+        <v>12447</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1025</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -6043,11 +6043,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>12714</v>
+        <v>12764</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+913</t>
+          <t>+963</t>
         </is>
       </c>
     </row>
@@ -6073,11 +6073,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>6876</v>
+        <v>6886</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+474</t>
+          <t>+484</t>
         </is>
       </c>
     </row>
@@ -6088,11 +6088,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>6833</v>
+        <v>6858</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+487</t>
+          <t>+512</t>
         </is>
       </c>
     </row>
@@ -6103,11 +6103,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>6806</v>
+        <v>6831</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+505</t>
+          <t>+530</t>
         </is>
       </c>
     </row>
@@ -6133,11 +6133,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>11160</v>
+        <v>11210</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+885</t>
+          <t>+935</t>
         </is>
       </c>
     </row>
@@ -6148,11 +6148,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>12108</v>
+        <v>12158</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+967</t>
+          <t>+1017</t>
         </is>
       </c>
     </row>
@@ -6163,11 +6163,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>11854</v>
+        <v>11904</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+975</t>
+          <t>+1025</t>
         </is>
       </c>
     </row>
@@ -6178,11 +6178,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>10467</v>
+        <v>10517</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+901</t>
+          <t>+951</t>
         </is>
       </c>
     </row>
@@ -6298,11 +6298,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>6770</v>
+        <v>6795</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+481</t>
+          <t>+506</t>
         </is>
       </c>
     </row>
@@ -6388,11 +6388,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>3471</v>
+        <v>3496</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+976</t>
+          <t>+1001</t>
         </is>
       </c>
     </row>
@@ -6403,11 +6403,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>3422</v>
+        <v>3447</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+972</t>
+          <t>+997</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -6595,7 +6595,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:01:00</t>
+          <t>Timestamp: 2026-07-30 13:31:00</t>
         </is>
       </c>
     </row>
@@ -6818,11 +6818,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>13491</v>
+        <v>13516</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1044</t>
+          <t>+1069</t>
         </is>
       </c>
     </row>
@@ -6938,11 +6938,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>7145</v>
+        <v>7220</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+525</t>
         </is>
       </c>
     </row>
@@ -6953,11 +6953,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>7336</v>
+        <v>7411</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+525</t>
         </is>
       </c>
     </row>
@@ -6968,11 +6968,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>7308</v>
+        <v>7383</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+525</t>
         </is>
       </c>
     </row>
@@ -6983,11 +6983,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>7281</v>
+        <v>7356</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+525</t>
         </is>
       </c>
     </row>
@@ -6998,11 +6998,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2197</v>
+        <v>2239</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+460</t>
+          <t>+502</t>
         </is>
       </c>
     </row>
@@ -7178,11 +7178,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>7245</v>
+        <v>7292</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+497</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -23,6 +23,7 @@
     <sheet name="2026-07-28" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-07-29" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-07-30" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026-07-31" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7450,6 +7451,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-31 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>10696</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+827</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>11026</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>11029</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>10662</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+696</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>10299</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+672</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10300</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+647</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>11659</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>11249</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>11032</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>10893</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>10701</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2248</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1702</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>14241</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>9918</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+655</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>12231</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+631</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11801</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+623</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>11520</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>11381</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+651</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>11022</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>14503</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+709</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7618</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+398</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7849</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+438</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>7809</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+426</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7782</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+426</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2364</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>12833</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>13875</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>13551</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+597</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>12060</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+543</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>831</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>827</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>646</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1743</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1701</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1589</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1462</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>7718</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+426</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1510</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>7593</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7546</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+378</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>7568</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>8117</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+949</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Minato Namikaze</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5063</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+641</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5065</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+668</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2499</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2346</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>2299</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2238</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2176</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4262</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+734</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>7818</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>The ArchitectX</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>1546</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>867</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+180</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -7475,7 +7475,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-31 13:01:00</t>
+          <t>Timestamp: 2026-07-31 13:31:00</t>
         </is>
       </c>
     </row>
@@ -7533,11 +7533,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>11026</v>
+        <v>11076</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+580</t>
+          <t>+630</t>
         </is>
       </c>
     </row>
@@ -7548,11 +7548,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>11029</v>
+        <v>11054</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+725</t>
         </is>
       </c>
     </row>
@@ -7563,11 +7563,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>10662</v>
+        <v>10687</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+696</t>
+          <t>+721</t>
         </is>
       </c>
     </row>
@@ -7578,11 +7578,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>10299</v>
+        <v>10324</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+672</t>
+          <t>+697</t>
         </is>
       </c>
     </row>
@@ -7593,11 +7593,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>10300</v>
+        <v>10325</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+647</t>
+          <t>+672</t>
         </is>
       </c>
     </row>
@@ -7608,11 +7608,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>11659</v>
+        <v>11709</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>11249</v>
+        <v>11299</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -7638,11 +7638,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>11032</v>
+        <v>11057</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+605</t>
+          <t>+630</t>
         </is>
       </c>
     </row>
@@ -7653,11 +7653,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>10893</v>
+        <v>10918</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -7668,11 +7668,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>10701</v>
+        <v>10726</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -7683,11 +7683,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>2248</v>
+        <v>2273</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1702</t>
+          <t>+1727</t>
         </is>
       </c>
     </row>
@@ -7698,11 +7698,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>14241</v>
+        <v>14266</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+725</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -7728,11 +7728,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>12231</v>
+        <v>12281</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+631</t>
+          <t>+681</t>
         </is>
       </c>
     </row>
@@ -7743,11 +7743,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>11801</v>
+        <v>11851</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+623</t>
+          <t>+673</t>
         </is>
       </c>
     </row>
@@ -7758,11 +7758,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>11520</v>
+        <v>11570</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+725</t>
         </is>
       </c>
     </row>
@@ -7773,11 +7773,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>11381</v>
+        <v>11431</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+651</t>
+          <t>+701</t>
         </is>
       </c>
     </row>
@@ -7788,11 +7788,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>11022</v>
+        <v>11072</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+599</t>
+          <t>+649</t>
         </is>
       </c>
     </row>
@@ -7803,11 +7803,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>14503</v>
+        <v>14528</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+709</t>
+          <t>+734</t>
         </is>
       </c>
     </row>
@@ -7878,11 +7878,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2364</v>
+        <v>2389</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -7893,11 +7893,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>12833</v>
+        <v>12858</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
@@ -7908,11 +7908,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>13875</v>
+        <v>13900</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
@@ -7923,11 +7923,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>13551</v>
+        <v>13577</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+597</t>
+          <t>+623</t>
         </is>
       </c>
     </row>
@@ -7938,11 +7938,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>12060</v>
+        <v>12065</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+548</t>
         </is>
       </c>
     </row>
@@ -7998,11 +7998,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>1743</v>
+        <v>1768</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8013,11 +8013,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>1701</v>
+        <v>1726</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8028,11 +8028,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>1589</v>
+        <v>1614</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8043,11 +8043,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>1462</v>
+        <v>1487</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8073,11 +8073,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>1510</v>
+        <v>1535</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+100</t>
+          <t>+125</t>
         </is>
       </c>
     </row>
@@ -8148,11 +8148,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>5063</v>
+        <v>5088</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+641</t>
+          <t>+666</t>
         </is>
       </c>
     </row>
@@ -8178,11 +8178,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>2499</v>
+        <v>2524</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8193,11 +8193,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>2346</v>
+        <v>2371</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8208,11 +8208,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>2299</v>
+        <v>2324</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8223,11 +8223,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>2238</v>
+        <v>2258</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+125</t>
+          <t>+145</t>
         </is>
       </c>
     </row>
@@ -8238,11 +8238,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>2176</v>
+        <v>2201</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+100</t>
+          <t>+125</t>
         </is>
       </c>
     </row>
@@ -8298,11 +8298,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>867</v>
+        <v>942</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+75</t>
+          <t>+150</t>
         </is>
       </c>
     </row>
@@ -8313,11 +8313,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>2006</v>
+        <v>2106</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+180</t>
+          <t>+280</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -8355,7 +8355,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-01 13:01:00</t>
+          <t>Timestamp: 2026-08-01 13:31:00</t>
         </is>
       </c>
     </row>
@@ -9133,11 +9133,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>4631</v>
+        <v>4674</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+369</t>
+          <t>+412</t>
         </is>
       </c>
     </row>
@@ -9193,11 +9193,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>2206</v>
+        <v>2388</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+100</t>
+          <t>+282</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -25,6 +25,7 @@
     <sheet name="2026-07-30" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-07-31" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-08-01" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2026-08-02" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9210,6 +9211,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-02 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>12950</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1683</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>12034</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>11791</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>11492</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>11149</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>11150</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>12699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>12299</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>12057</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>11927</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>11735</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2273</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1627</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>15771</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>10768</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>13301</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>12876</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>12579</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>12456</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>12085</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>15561</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>8668</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>8899</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8859</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8782</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2389</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>13792</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>14876</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>14521</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+169</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>12981</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+96</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>831</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>827</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>646</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1843</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1801</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1689</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1562</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8698</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1610</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>8592</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-33</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>8646</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+21</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>8668</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>9267</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+642</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Minato Namikaze</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5861</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5915</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2574</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2421</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>2374</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2313</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2251</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>5406</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+732</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>8817</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+192</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>The ArchitectX</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>1546</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>2779</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+391</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -9235,7 +9235,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-02 13:01:00</t>
+          <t>Timestamp: 2026-08-02 13:31:00</t>
         </is>
       </c>
     </row>
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>2779</v>
+        <v>2961</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+391</t>
+          <t>+573</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -10994,7 +10994,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-03 13:01:00</t>
+          <t>Timestamp: 2026-08-03 13:31:00</t>
         </is>
       </c>
     </row>
@@ -11337,11 +11337,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>10284</v>
+        <v>10309</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1616</t>
+          <t>+1641</t>
         </is>
       </c>
     </row>
@@ -11352,11 +11352,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>10560</v>
+        <v>10585</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1661</t>
+          <t>+1686</t>
         </is>
       </c>
     </row>
@@ -11367,11 +11367,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>10664</v>
+        <v>10689</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1805</t>
+          <t>+1830</t>
         </is>
       </c>
     </row>
@@ -11382,11 +11382,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>10587</v>
+        <v>10612</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1805</t>
+          <t>+1830</t>
         </is>
       </c>
     </row>
@@ -11577,11 +11577,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>10408</v>
+        <v>10433</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1710</t>
+          <t>+1735</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -11874,7 +11874,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-04 13:01:00</t>
+          <t>Timestamp: 2026-08-04 13:31:00</t>
         </is>
       </c>
     </row>
@@ -12217,11 +12217,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>11444</v>
+        <v>11469</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1135</t>
+          <t>+1160</t>
         </is>
       </c>
     </row>
@@ -12232,11 +12232,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>11700</v>
+        <v>11725</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1115</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -12247,11 +12247,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>11840</v>
+        <v>11865</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1151</t>
+          <t>+1176</t>
         </is>
       </c>
     </row>
@@ -12262,11 +12262,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>11739</v>
+        <v>11764</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1127</t>
+          <t>+1152</t>
         </is>
       </c>
     </row>
@@ -12457,11 +12457,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>11592</v>
+        <v>11617</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1159</t>
+          <t>+1184</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -12754,7 +12754,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-05 13:01:00</t>
+          <t>Timestamp: 2026-08-05 13:31:00</t>
         </is>
       </c>
     </row>
@@ -13097,11 +13097,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>12854</v>
+        <v>12904</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1385</t>
+          <t>+1435</t>
         </is>
       </c>
     </row>
@@ -13112,11 +13112,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>13035</v>
+        <v>13085</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1310</t>
+          <t>+1360</t>
         </is>
       </c>
     </row>
@@ -13127,11 +13127,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>13238</v>
+        <v>13288</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1373</t>
+          <t>+1423</t>
         </is>
       </c>
     </row>
@@ -13142,11 +13142,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>13164</v>
+        <v>13214</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+1450</t>
         </is>
       </c>
     </row>
@@ -13337,11 +13337,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>12972</v>
+        <v>13022</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1355</t>
+          <t>+1405</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -14514,7 +14514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:01:00</t>
+          <t>Timestamp: 2026-08-07 13:31:00</t>
         </is>
       </c>
     </row>
@@ -14872,11 +14872,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>16857</v>
+        <v>16877</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1431</t>
+          <t>+1451</t>
         </is>
       </c>
     </row>
@@ -14887,11 +14887,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>16975</v>
+        <v>17125</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1382</t>
+          <t>+1532</t>
         </is>
       </c>
     </row>
@@ -14902,11 +14902,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>16928</v>
+        <v>17078</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+1550</t>
         </is>
       </c>
     </row>
@@ -15097,11 +15097,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>16745</v>
+        <v>16895</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1400</t>
+          <t>+1550</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-09 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -32,6 +32,7 @@
     <sheet name="2026-08-06" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026-08-09" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16249,6 +16250,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-09 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>25425</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+3100</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>12034</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>11791</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>11492</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>11149</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>11150</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>12699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>12299</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>12057</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>11927</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>11735</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2273</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1627</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>18153</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>10768</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>13301</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>12876</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>12579</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>12456</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>12085</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>15961</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>19191</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>19318</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>19521</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>19501</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2389</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>14092</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>15276</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>14921</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>13281</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>831</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>827</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>646</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1843</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1801</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>1689</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1562</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>19345</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1610</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>8592</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-225</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>8646</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-171</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>8668</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>9267</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Minato Namikaze</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5861</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5915</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2574</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2421</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>2374</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2313</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2251</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>6606</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>8817</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>CP9 ArchitectX</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>2593</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>1682</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>5813</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -17154,7 +17154,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-10 13:01:00</t>
+          <t>Timestamp: 2026-08-10 13:31:00</t>
         </is>
       </c>
     </row>
@@ -17932,11 +17932,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>0</v>
+        <v>1375</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>-1682</t>
+          <t>-307</t>
         </is>
       </c>
     </row>
@@ -17962,7 +17962,7 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>428</v>
+        <v>553</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
@@ -17977,7 +17977,7 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>420</v>
+        <v>545</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
@@ -17992,7 +17992,7 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>420</v>
+        <v>545</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -21553,7 +21553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-14 13:01:00</t>
+          <t>Timestamp: 2026-08-14 13:31:00</t>
         </is>
       </c>
     </row>
@@ -21896,11 +21896,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1375</v>
+        <v>1500</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1375</t>
+          <t>+1500</t>
         </is>
       </c>
     </row>
@@ -21911,11 +21911,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1375</v>
+        <v>1500</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1375</t>
+          <t>+1500</t>
         </is>
       </c>
     </row>
@@ -21926,11 +21926,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1375</v>
+        <v>1500</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1375</t>
+          <t>+1500</t>
         </is>
       </c>
     </row>
@@ -21941,11 +21941,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1375</v>
+        <v>1500</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1375</t>
+          <t>+1500</t>
         </is>
       </c>
     </row>
@@ -22136,11 +22136,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>1375</v>
+        <v>1500</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1375</t>
+          <t>+1500</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -22433,7 +22433,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-15 13:01:00</t>
+          <t>Timestamp: 2026-08-15 13:31:00</t>
         </is>
       </c>
     </row>
@@ -22491,11 +22491,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4876</v>
+        <v>5156</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+2730</t>
+          <t>+3010</t>
         </is>
       </c>
     </row>
@@ -22506,11 +22506,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>700</v>
+        <v>1120</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -22521,11 +22521,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>700</v>
+        <v>1120</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -22536,11 +22536,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>700</v>
+        <v>1120</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -22551,11 +22551,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>700</v>
+        <v>1120</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -22566,11 +22566,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>5005</v>
+        <v>5285</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+2628</t>
+          <t>+2908</t>
         </is>
       </c>
     </row>
@@ -22581,11 +22581,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4737</v>
+        <v>5017</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+2730</t>
+          <t>+3010</t>
         </is>
       </c>
     </row>
@@ -22596,11 +22596,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5005</v>
+        <v>5285</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+2730</t>
+          <t>+3010</t>
         </is>
       </c>
     </row>
@@ -22611,11 +22611,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>4793</v>
+        <v>5073</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+2686</t>
+          <t>+2966</t>
         </is>
       </c>
     </row>
@@ -22626,11 +22626,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>4949</v>
+        <v>5229</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2670</t>
+          <t>+2950</t>
         </is>
       </c>
     </row>
@@ -22656,11 +22656,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>6941</v>
+        <v>7081</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+2980</t>
+          <t>+3120</t>
         </is>
       </c>
     </row>
@@ -22671,11 +22671,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>720</v>
+        <v>1140</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -22686,11 +22686,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>3505</v>
+        <v>3645</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1520</t>
         </is>
       </c>
     </row>
@@ -22701,11 +22701,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>3270</v>
+        <v>3410</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1520</t>
         </is>
       </c>
     </row>
@@ -22716,11 +22716,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>3606</v>
+        <v>3746</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1356</t>
+          <t>+1496</t>
         </is>
       </c>
     </row>
@@ -22731,11 +22731,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>3422</v>
+        <v>3562</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1340</t>
+          <t>+1480</t>
         </is>
       </c>
     </row>
@@ -22746,11 +22746,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3138</v>
+        <v>3278</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -22761,11 +22761,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1329</v>
+        <v>1889</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+1530</t>
         </is>
       </c>
     </row>
@@ -22776,11 +22776,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>3748</v>
+        <v>3888</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2248</t>
+          <t>+2388</t>
         </is>
       </c>
     </row>
@@ -22791,11 +22791,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>3515</v>
+        <v>3655</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2015</t>
+          <t>+2155</t>
         </is>
       </c>
     </row>
@@ -22806,11 +22806,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>3521</v>
+        <v>3661</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2021</t>
+          <t>+2161</t>
         </is>
       </c>
     </row>
@@ -22821,11 +22821,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>3675</v>
+        <v>3815</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+2175</t>
+          <t>+2315</t>
         </is>
       </c>
     </row>
@@ -22851,11 +22851,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1090</v>
+        <v>1510</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+1210</t>
         </is>
       </c>
     </row>
@@ -22866,11 +22866,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1170</v>
+        <v>1730</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+970</t>
+          <t>+1530</t>
         </is>
       </c>
     </row>
@@ -22881,11 +22881,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1010</v>
+        <v>1570</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+810</t>
+          <t>+1370</t>
         </is>
       </c>
     </row>
@@ -22896,11 +22896,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1140</v>
+        <v>1560</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+720</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -23016,11 +23016,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3560</v>
+        <v>3700</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+2060</t>
+          <t>+2200</t>
         </is>
       </c>
     </row>
@@ -23046,11 +23046,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>1090</v>
+        <v>1230</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1090</t>
+          <t>+1230</t>
         </is>
       </c>
     </row>
@@ -23061,11 +23061,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>1000</v>
+        <v>1140</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -23076,11 +23076,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>1000</v>
+        <v>1140</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -23091,11 +23091,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>1140</v>
+        <v>1280</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1280</t>
         </is>
       </c>
     </row>
@@ -23196,11 +23196,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>1140</v>
+        <v>1280</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+1140</t>
+          <t>+1280</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -39,6 +39,7 @@
     <sheet name="2026-08-13" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-08-14" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-15" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="2026-08-16" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23288,6 +23289,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-16 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>18756</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+3100</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>8876</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+3720</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2980</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1860</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>2980</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1860</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>2980</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1860</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2980</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1860</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>9005</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+3720</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>8575</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+3558</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>8808</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+3523</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>8434</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+3361</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>8582</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+3353</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>12032</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+4951</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1860</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>8228</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+4583</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8050</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+4640</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>8378</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+4632</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7902</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+4340</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7226</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+3948</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>5849</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+3960</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>7714</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+3826</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7535</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+3880</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>7514</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+3853</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7560</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+3745</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>5063</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+3553</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>5542</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+3812</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>5230</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+3660</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>4407</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+2847</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>7445</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+3745</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>5752</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+4472</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>5660</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+4380</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>5660</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+4520</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>5929</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+4649</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6734</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>5820</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+4540</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4295</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>5319</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1493</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>3746</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>-159</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3865</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>3905</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -24193,7 +24193,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:01:00</t>
+          <t>Timestamp: 2026-08-17 13:31:00</t>
         </is>
       </c>
     </row>
@@ -24251,11 +24251,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>13495</v>
+        <v>13520</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+4619</t>
+          <t>+4644</t>
         </is>
       </c>
     </row>
@@ -24326,11 +24326,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>11513</v>
+        <v>11538</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+2508</t>
+          <t>+2533</t>
         </is>
       </c>
     </row>
@@ -24341,11 +24341,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>11034</v>
+        <v>11059</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+2459</t>
+          <t>+2484</t>
         </is>
       </c>
     </row>
@@ -24356,11 +24356,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>11338</v>
+        <v>11363</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+2530</t>
+          <t>+2555</t>
         </is>
       </c>
     </row>
@@ -24371,11 +24371,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>20328</v>
+        <v>20353</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+11894</t>
+          <t>+11919</t>
         </is>
       </c>
     </row>
@@ -24386,11 +24386,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>34363</v>
+        <v>34388</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+25781</t>
+          <t>+25806</t>
         </is>
       </c>
     </row>
@@ -24806,11 +24806,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>9072</v>
+        <v>9097</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+3252</t>
+          <t>+3277</t>
         </is>
       </c>
     </row>
@@ -24821,11 +24821,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>8860</v>
+        <v>8885</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+3040</t>
+          <t>+3065</t>
         </is>
       </c>
     </row>
@@ -24836,11 +24836,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>8440</v>
+        <v>8465</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+2780</t>
+          <t>+2805</t>
         </is>
       </c>
     </row>
@@ -24851,11 +24851,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>8971</v>
+        <v>8996</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+3151</t>
+          <t>+3176</t>
         </is>
       </c>
     </row>
@@ -24941,11 +24941,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>7414</v>
+        <v>7514</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+780</t>
         </is>
       </c>
     </row>
@@ -24956,11 +24956,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>37707</v>
+        <v>37732</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+31887</t>
+          <t>+31912</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -41,6 +41,7 @@
     <sheet name="2026-08-15" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="2026-08-16" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-17" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="2026-08-18" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25048,6 +25049,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-18 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>22826</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+656</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>15589</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+2069</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3700</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3700</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>3700</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>3620</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>12388</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>11909</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>12156</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+793</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>21178</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>35213</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>16613</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3600</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10988</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>10470</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10998</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>10446</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>13608</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8883</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>9339</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>9160</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>9139</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>9185</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7857</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8552</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8071</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>38748</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>9070</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>9747</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-27985</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>9519</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-28213</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>9115</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>9643</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-28089</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>7889</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>38379</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+647</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4295</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>6019</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>3746</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>-159</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3865</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>3905</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -25073,7 +25073,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-18 13:01:00</t>
+          <t>Timestamp: 2026-08-18 13:31:00</t>
         </is>
       </c>
     </row>
@@ -25131,11 +25131,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>15589</v>
+        <v>15639</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+2069</t>
+          <t>+2119</t>
         </is>
       </c>
     </row>
@@ -25206,11 +25206,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>12388</v>
+        <v>12438</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -25416,11 +25416,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>9339</v>
+        <v>9364</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25431,11 +25431,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>9160</v>
+        <v>9185</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25446,11 +25446,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>9139</v>
+        <v>9164</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25461,11 +25461,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>9185</v>
+        <v>9210</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25656,11 +25656,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>9070</v>
+        <v>9095</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -25953,7 +25953,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:01:00</t>
+          <t>Timestamp: 2026-08-19 13:31:00</t>
         </is>
       </c>
     </row>
@@ -26011,11 +26011,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>16729</v>
+        <v>16829</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1090</t>
+          <t>+1190</t>
         </is>
       </c>
     </row>
@@ -26296,11 +26296,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>10169</v>
+        <v>10219</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+805</t>
+          <t>+855</t>
         </is>
       </c>
     </row>
@@ -26311,11 +26311,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>10010</v>
+        <v>10060</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -26326,11 +26326,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>9981</v>
+        <v>10031</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+817</t>
+          <t>+867</t>
         </is>
       </c>
     </row>
@@ -26341,11 +26341,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>10035</v>
+        <v>10108</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+898</t>
         </is>
       </c>
     </row>
@@ -26536,11 +26536,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>9920</v>
+        <v>9930</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+835</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 13:01:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -43,6 +43,7 @@
     <sheet name="2026-08-17" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-18" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-19" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="2026-08-20" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26808,6 +26809,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-20 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24986</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>18579</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1750</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3700</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3700</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>3700</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>3620</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>15411</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1850</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>14959</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1850</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>15170</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1823</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>24117</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>38170</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1782</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>19554</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1741</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3600</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>11388</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>10870</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>11389</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+391</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>10796</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>13958</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8883</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>11924</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1705</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>11765</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1705</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>11633</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1602</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>11658</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1550</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7857</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8552</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8071</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>38748</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1604</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>9747</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-28632</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>9519</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-28860</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>9115</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>9643</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-28736</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Last Ninjas</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Mahogakure</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>7989</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>38379</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4520</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>6419</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>3746</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>-159</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3865</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>3905</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 13:31:00
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -26833,7 +26833,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:01:00</t>
+          <t>Timestamp: 2026-08-20 13:31:00</t>
         </is>
       </c>
     </row>
@@ -27206,11 +27206,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>11633</v>
+        <v>11637</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1602</t>
+          <t>+1606</t>
         </is>
       </c>
     </row>
@@ -27221,11 +27221,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>11658</v>
+        <v>11808</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1550</t>
+          <t>+1700</t>
         </is>
       </c>
     </row>
@@ -27416,11 +27416,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>11534</v>
+        <v>11684</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1604</t>
+          <t>+1754</t>
         </is>
       </c>
     </row>
@@ -27626,11 +27626,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>6419</v>
+        <v>6619</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+200</t>
+          <t>+400</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -44,6 +44,7 @@
     <sheet name="2026-08-18" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-19" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-20" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026-08-21" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27688,6 +27689,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-21 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>26227</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1241</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>19404</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4175</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+475</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>4175</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+475</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4116</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+416</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>4045</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>16336</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>15834</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>15895</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>24842</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>38895</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>21059</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1505</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4025</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>12700</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1312</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>12159</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1289</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>12714</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1325</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>12121</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1325</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>15283</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1325</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>9363</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>12489</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+565</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>12377</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+612</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>12337</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>12508</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8257</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8521</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>39153</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+405</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sakura</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Î·Î±mÃ¯Ã¯Ã¯ Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Å¡hÃ¯ÎºÎ±mÎ±ru Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>12384</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>uÎ·ÎºÎ·Ã¸Ï‰Î· Î·Ã¸Ã¯r</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>10147</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-28232</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>9936</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-28443</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>9540</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>10118</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-28261</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Emblem Elite</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>8389</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>38854</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+475</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>4520</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>7019</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4921</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1016</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>5040</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>5072</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+1167</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -27713,7 +27713,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:01:00</t>
+          <t>Timestamp: 2026-08-21 13:31:00</t>
         </is>
       </c>
     </row>
@@ -27771,11 +27771,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>19404</v>
+        <v>19429</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+850</t>
         </is>
       </c>
     </row>
@@ -27786,11 +27786,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>4175</v>
+        <v>4200</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+500</t>
         </is>
       </c>
     </row>
@@ -27801,11 +27801,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>4175</v>
+        <v>4200</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+500</t>
         </is>
       </c>
     </row>
@@ -27816,11 +27816,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>4116</v>
+        <v>4141</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+416</t>
+          <t>+441</t>
         </is>
       </c>
     </row>
@@ -27831,11 +27831,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>4045</v>
+        <v>4070</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+450</t>
         </is>
       </c>
     </row>
@@ -27936,11 +27936,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>21059</v>
+        <v>21109</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1505</t>
+          <t>+1555</t>
         </is>
       </c>
     </row>
@@ -27951,11 +27951,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>4025</v>
+        <v>4050</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+450</t>
         </is>
       </c>
     </row>
@@ -27966,11 +27966,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>12700</v>
+        <v>12705</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1312</t>
+          <t>+1317</t>
         </is>
       </c>
     </row>
@@ -27981,11 +27981,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>12159</v>
+        <v>12184</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1289</t>
+          <t>+1314</t>
         </is>
       </c>
     </row>
@@ -27996,11 +27996,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>12714</v>
+        <v>12739</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1325</t>
+          <t>+1350</t>
         </is>
       </c>
     </row>
@@ -28011,11 +28011,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>12121</v>
+        <v>12146</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1325</t>
+          <t>+1350</t>
         </is>
       </c>
     </row>
@@ -28026,11 +28026,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>15283</v>
+        <v>15308</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1325</t>
+          <t>+1350</t>
         </is>
       </c>
     </row>
@@ -28041,11 +28041,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>9363</v>
+        <v>9388</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+505</t>
         </is>
       </c>
     </row>
@@ -28131,11 +28131,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>8257</v>
+        <v>8282</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+425</t>
         </is>
       </c>
     </row>
@@ -28146,11 +28146,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>9002</v>
+        <v>9027</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -28161,11 +28161,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>8521</v>
+        <v>8546</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -28326,11 +28326,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>10147</v>
+        <v>10197</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>-28232</t>
+          <t>-28182</t>
         </is>
       </c>
     </row>
@@ -28341,11 +28341,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>9936</v>
+        <v>9961</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>-28443</t>
+          <t>-28418</t>
         </is>
       </c>
     </row>
@@ -28356,11 +28356,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>9540</v>
+        <v>9565</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+450</t>
         </is>
       </c>
     </row>
@@ -28371,11 +28371,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>10118</v>
+        <v>10143</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>-28261</t>
+          <t>-28236</t>
         </is>
       </c>
     </row>
@@ -28446,11 +28446,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>38854</v>
+        <v>38879</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+500</t>
         </is>
       </c>
     </row>
@@ -28491,11 +28491,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>4921</v>
+        <v>4946</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1016</t>
+          <t>+1041</t>
         </is>
       </c>
     </row>
@@ -28506,11 +28506,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>5040</v>
+        <v>5065</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -28521,11 +28521,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>5072</v>
+        <v>5097</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+1167</t>
+          <t>+1192</t>
         </is>
       </c>
     </row>
@@ -28536,7 +28536,7 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>225</v>
+        <v>250</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
@@ -28551,7 +28551,7 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>225</v>
+        <v>250</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -28593,7 +28593,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-22 13:01:00</t>
+          <t>Timestamp: 2026-08-22 13:31:00</t>
         </is>
       </c>
     </row>
@@ -28651,11 +28651,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>20119</v>
+        <v>20200</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+771</t>
         </is>
       </c>
     </row>
@@ -28666,11 +28666,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>4900</v>
+        <v>4950</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -28681,11 +28681,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>4900</v>
+        <v>4950</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -28696,11 +28696,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>4828</v>
+        <v>4878</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+687</t>
+          <t>+737</t>
         </is>
       </c>
     </row>
@@ -28711,11 +28711,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>4745</v>
+        <v>4795</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+725</t>
         </is>
       </c>
     </row>
@@ -28726,11 +28726,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>17036</v>
+        <v>17086</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -28741,11 +28741,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>16529</v>
+        <v>16579</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+695</t>
+          <t>+745</t>
         </is>
       </c>
     </row>
@@ -28756,11 +28756,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>16570</v>
+        <v>16620</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+725</t>
         </is>
       </c>
     </row>
@@ -28771,11 +28771,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>25502</v>
+        <v>25552</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+660</t>
+          <t>+710</t>
         </is>
       </c>
     </row>
@@ -28786,11 +28786,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>39540</v>
+        <v>39590</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+645</t>
+          <t>+695</t>
         </is>
       </c>
     </row>
@@ -28831,11 +28831,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>4725</v>
+        <v>4775</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+725</t>
         </is>
       </c>
     </row>
@@ -28846,11 +28846,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>13380</v>
+        <v>13480</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+775</t>
         </is>
       </c>
     </row>
@@ -28861,11 +28861,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>12848</v>
+        <v>12948</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+664</t>
+          <t>+764</t>
         </is>
       </c>
     </row>
@@ -28876,11 +28876,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>13389</v>
+        <v>13489</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+650</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -28891,11 +28891,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>12780</v>
+        <v>12880</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+634</t>
+          <t>+734</t>
         </is>
       </c>
     </row>
@@ -28906,11 +28906,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>15913</v>
+        <v>16013</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+605</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -28921,11 +28921,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>10018</v>
+        <v>10068</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+630</t>
+          <t>+680</t>
         </is>
       </c>
     </row>
@@ -29011,11 +29011,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>8857</v>
+        <v>8907</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -29026,11 +29026,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>9632</v>
+        <v>9682</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+605</t>
+          <t>+655</t>
         </is>
       </c>
     </row>
@@ -29041,11 +29041,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>9151</v>
+        <v>9201</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+605</t>
+          <t>+655</t>
         </is>
       </c>
     </row>
@@ -29056,11 +29056,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>39716</v>
+        <v>39766</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+563</t>
+          <t>+613</t>
         </is>
       </c>
     </row>
@@ -29206,11 +29206,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>10947</v>
+        <v>10997</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>-27932</t>
+          <t>-27882</t>
         </is>
       </c>
     </row>
@@ -29221,11 +29221,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>10711</v>
+        <v>10761</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>-28168</t>
+          <t>-28118</t>
         </is>
       </c>
     </row>
@@ -29236,11 +29236,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>10275</v>
+        <v>10325</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+710</t>
+          <t>+760</t>
         </is>
       </c>
     </row>
@@ -29251,11 +29251,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>10935</v>
+        <v>10985</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>-27944</t>
+          <t>-27894</t>
         </is>
       </c>
     </row>
@@ -29326,11 +29326,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>39538</v>
+        <v>39588</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+659</t>
+          <t>+709</t>
         </is>
       </c>
     </row>
@@ -29371,11 +29371,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>6046</v>
+        <v>6096</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+949</t>
+          <t>+999</t>
         </is>
       </c>
     </row>
@@ -29386,11 +29386,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>6161</v>
+        <v>6211</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+1096</t>
+          <t>+1146</t>
         </is>
       </c>
     </row>
@@ -29401,11 +29401,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>6192</v>
+        <v>6242</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+1095</t>
+          <t>+1145</t>
         </is>
       </c>
     </row>
@@ -29416,11 +29416,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>1256</v>
+        <v>1306</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+1006</t>
+          <t>+1056</t>
         </is>
       </c>
     </row>
@@ -29431,11 +29431,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>1300</v>
+        <v>1314</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1064</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -30352,7 +30352,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:01:00</t>
+          <t>Timestamp: 2026-08-23 13:31:00</t>
         </is>
       </c>
     </row>
@@ -30425,11 +30425,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>7172</v>
+        <v>7222</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+2222</t>
+          <t>+2272</t>
         </is>
       </c>
     </row>
@@ -30440,11 +30440,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>14176</v>
+        <v>14226</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+9226</t>
+          <t>+9276</t>
         </is>
       </c>
     </row>
@@ -30455,11 +30455,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>7075</v>
+        <v>7125</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+2197</t>
+          <t>+2247</t>
         </is>
       </c>
     </row>
@@ -30470,11 +30470,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7055</v>
+        <v>7105</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+2260</t>
+          <t>+2310</t>
         </is>
       </c>
     </row>
@@ -30515,11 +30515,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>18210</v>
+        <v>18230</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1590</t>
+          <t>+1610</t>
         </is>
       </c>
     </row>
@@ -30530,11 +30530,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>27123</v>
+        <v>27223</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1571</t>
+          <t>+1671</t>
         </is>
       </c>
     </row>
@@ -30545,11 +30545,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>41153</v>
+        <v>41253</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1563</t>
+          <t>+1663</t>
         </is>
       </c>
     </row>
@@ -30590,11 +30590,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>9106</v>
+        <v>9156</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+4331</t>
+          <t>+4381</t>
         </is>
       </c>
     </row>
@@ -30605,11 +30605,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>15570</v>
+        <v>15690</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+2090</t>
+          <t>+2210</t>
         </is>
       </c>
     </row>
@@ -30620,11 +30620,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>15111</v>
+        <v>15231</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+2163</t>
+          <t>+2283</t>
         </is>
       </c>
     </row>
@@ -30635,11 +30635,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>15665</v>
+        <v>15785</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2176</t>
+          <t>+2296</t>
         </is>
       </c>
     </row>
@@ -30650,11 +30650,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>20165</v>
+        <v>20285</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+7285</t>
+          <t>+7405</t>
         </is>
       </c>
     </row>
@@ -30665,11 +30665,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>24142</v>
+        <v>24262</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+8129</t>
+          <t>+8249</t>
         </is>
       </c>
     </row>
@@ -30680,11 +30680,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>12344</v>
+        <v>12394</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2276</t>
+          <t>+2326</t>
         </is>
       </c>
     </row>
@@ -30695,11 +30695,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>14375</v>
+        <v>14425</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1486</t>
+          <t>+1536</t>
         </is>
       </c>
     </row>
@@ -30710,11 +30710,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>14327</v>
+        <v>14377</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1550</t>
+          <t>+1600</t>
         </is>
       </c>
     </row>
@@ -30725,11 +30725,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>14267</v>
+        <v>14317</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1530</t>
+          <t>+1580</t>
         </is>
       </c>
     </row>
@@ -30740,11 +30740,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>14413</v>
+        <v>14463</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1505</t>
+          <t>+1555</t>
         </is>
       </c>
     </row>
@@ -30770,11 +30770,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>11158</v>
+        <v>11208</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+2251</t>
+          <t>+2301</t>
         </is>
       </c>
     </row>
@@ -30785,11 +30785,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>11851</v>
+        <v>11901</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2169</t>
+          <t>+2219</t>
         </is>
       </c>
     </row>
@@ -30815,11 +30815,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>41974</v>
+        <v>42024</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2208</t>
+          <t>+2258</t>
         </is>
       </c>
     </row>
@@ -30830,11 +30830,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>691</v>
+        <v>780</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+691</t>
+          <t>+780</t>
         </is>
       </c>
     </row>
@@ -30935,11 +30935,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>26662</v>
+        <v>26712</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+13878</t>
+          <t>+13928</t>
         </is>
       </c>
     </row>
@@ -30965,11 +30965,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>13150</v>
+        <v>13200</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>-26438</t>
+          <t>-26388</t>
         </is>
       </c>
     </row>
@@ -30980,11 +30980,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>18248</v>
+        <v>18298</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>-21340</t>
+          <t>-21290</t>
         </is>
       </c>
     </row>
@@ -30995,11 +30995,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>16952</v>
+        <v>17002</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+6627</t>
+          <t>+6677</t>
         </is>
       </c>
     </row>
@@ -31010,11 +31010,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>13195</v>
+        <v>13245</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>-26393</t>
+          <t>-26343</t>
         </is>
       </c>
     </row>
@@ -31085,11 +31085,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>41778</v>
+        <v>41828</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+2190</t>
+          <t>+2240</t>
         </is>
       </c>
     </row>
@@ -31130,11 +31130,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>8447</v>
+        <v>8497</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+2205</t>
+          <t>+2255</t>
         </is>
       </c>
     </row>
@@ -31145,11 +31145,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>8498</v>
+        <v>8548</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+2287</t>
+          <t>+2337</t>
         </is>
       </c>
     </row>
@@ -31160,11 +31160,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>8502</v>
+        <v>8552</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+2260</t>
+          <t>+2310</t>
         </is>
       </c>
     </row>
@@ -31175,11 +31175,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>3656</v>
+        <v>3706</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -31190,11 +31190,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>3646</v>
+        <v>3696</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+2332</t>
+          <t>+2382</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -31232,7 +31232,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:01:00</t>
+          <t>Timestamp: 2026-08-24 13:31:00</t>
         </is>
       </c>
     </row>
@@ -31485,11 +31485,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>17946</v>
+        <v>17996</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+2256</t>
+          <t>+2306</t>
         </is>
       </c>
     </row>
@@ -31500,11 +31500,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>17463</v>
+        <v>17513</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+2232</t>
+          <t>+2282</t>
         </is>
       </c>
     </row>
@@ -31515,11 +31515,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>17910</v>
+        <v>17960</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2125</t>
+          <t>+2175</t>
         </is>
       </c>
     </row>
@@ -31530,11 +31530,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>22176</v>
+        <v>22226</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1891</t>
+          <t>+1941</t>
         </is>
       </c>
     </row>
@@ -31545,11 +31545,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>26435</v>
+        <v>26460</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2173</t>
+          <t>+2198</t>
         </is>
       </c>
     </row>
@@ -31845,11 +31845,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>14390</v>
+        <v>14440</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>-27438</t>
+          <t>-27388</t>
         </is>
       </c>
     </row>
@@ -31860,11 +31860,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>19452</v>
+        <v>19502</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>-22376</t>
+          <t>-22326</t>
         </is>
       </c>
     </row>
@@ -31875,11 +31875,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>18087</v>
+        <v>18137</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1085</t>
+          <t>+1135</t>
         </is>
       </c>
     </row>
@@ -31890,11 +31890,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>14460</v>
+        <v>14510</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>-27368</t>
+          <t>-27318</t>
         </is>
       </c>
     </row>
@@ -31965,11 +31965,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>42958</v>
+        <v>43008</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+1130</t>
+          <t>+1180</t>
         </is>
       </c>
     </row>
@@ -32010,11 +32010,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>10592</v>
+        <v>10617</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+2040</t>
+          <t>+2065</t>
         </is>
       </c>
     </row>
@@ -32025,11 +32025,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>10591</v>
+        <v>10616</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+2043</t>
+          <t>+2068</t>
         </is>
       </c>
     </row>
@@ -32040,11 +32040,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>10663</v>
+        <v>10688</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+2111</t>
+          <t>+2136</t>
         </is>
       </c>
     </row>
@@ -32055,11 +32055,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>5733</v>
+        <v>5758</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+2027</t>
+          <t>+2052</t>
         </is>
       </c>
     </row>
@@ -32070,11 +32070,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>5611</v>
+        <v>5636</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+1915</t>
+          <t>+1940</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -32112,7 +32112,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:01:00</t>
+          <t>Timestamp: 2026-08-25 13:31:00</t>
         </is>
       </c>
     </row>
@@ -32185,11 +32185,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>8496</v>
+        <v>8521</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+450</t>
         </is>
       </c>
     </row>
@@ -32200,11 +32200,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>15543</v>
+        <v>15568</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+450</t>
         </is>
       </c>
     </row>
@@ -32215,11 +32215,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8325</v>
+        <v>8350</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+380</t>
+          <t>+405</t>
         </is>
       </c>
     </row>
@@ -32230,11 +32230,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>8247</v>
+        <v>8272</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+425</t>
         </is>
       </c>
     </row>
@@ -32350,11 +32350,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>10290</v>
+        <v>10315</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+425</t>
         </is>
       </c>
     </row>
@@ -32365,11 +32365,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>18975</v>
+        <v>19050</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+979</t>
+          <t>+1054</t>
         </is>
       </c>
     </row>
@@ -32380,11 +32380,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>18544</v>
+        <v>18619</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1031</t>
+          <t>+1106</t>
         </is>
       </c>
     </row>
@@ -32395,11 +32395,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>19023</v>
+        <v>19098</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1063</t>
+          <t>+1138</t>
         </is>
       </c>
     </row>
@@ -32410,11 +32410,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>23331</v>
+        <v>23356</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1105</t>
+          <t>+1130</t>
         </is>
       </c>
     </row>
@@ -32425,11 +32425,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>27549</v>
+        <v>27574</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1089</t>
+          <t>+1114</t>
         </is>
       </c>
     </row>
@@ -32440,11 +32440,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>14065</v>
+        <v>14115</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+425</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -32530,11 +32530,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>12812</v>
+        <v>12862</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+450</t>
         </is>
       </c>
     </row>
@@ -32545,11 +32545,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>13557</v>
+        <v>13607</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+401</t>
+          <t>+451</t>
         </is>
       </c>
     </row>
@@ -32560,11 +32560,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>13094</v>
+        <v>13144</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+397</t>
+          <t>+447</t>
         </is>
       </c>
     </row>
@@ -32575,11 +32575,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>43718</v>
+        <v>43768</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+375</t>
+          <t>+425</t>
         </is>
       </c>
     </row>
@@ -32725,11 +32725,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>15583</v>
+        <v>15608</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>-27425</t>
+          <t>-27400</t>
         </is>
       </c>
     </row>
@@ -32740,11 +32740,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>20658</v>
+        <v>20683</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>-22350</t>
+          <t>-22325</t>
         </is>
       </c>
     </row>
@@ -32755,11 +32755,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>19292</v>
+        <v>19317</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1155</t>
+          <t>+1180</t>
         </is>
       </c>
     </row>
@@ -32770,11 +32770,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>15685</v>
+        <v>15710</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>-27323</t>
+          <t>-27298</t>
         </is>
       </c>
     </row>
@@ -32845,11 +32845,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>44183</v>
+        <v>44208</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -32992,7 +32992,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-26 13:01:00</t>
+          <t>Timestamp: 2026-08-26 13:31:00</t>
         </is>
       </c>
     </row>
@@ -33050,11 +33050,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>26005</v>
+        <v>26080</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+895</t>
+          <t>+970</t>
         </is>
       </c>
     </row>
@@ -33080,11 +33080,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>16448</v>
+        <v>16468</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -33095,11 +33095,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>9200</v>
+        <v>9275</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+925</t>
         </is>
       </c>
     </row>
@@ -33110,11 +33110,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>9122</v>
+        <v>9197</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+925</t>
         </is>
       </c>
     </row>
@@ -33140,11 +33140,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>22271</v>
+        <v>22346</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -33155,11 +33155,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>22307</v>
+        <v>22382</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+840</t>
+          <t>+915</t>
         </is>
       </c>
     </row>
@@ -33170,11 +33170,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>31230</v>
+        <v>31305</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+864</t>
+          <t>+939</t>
         </is>
       </c>
     </row>
@@ -33185,11 +33185,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>45278</v>
+        <v>45353</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+955</t>
         </is>
       </c>
     </row>
@@ -33215,11 +33215,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>25296</v>
+        <v>25421</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+375</t>
         </is>
       </c>
     </row>
@@ -33230,11 +33230,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>11161</v>
+        <v>11236</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+846</t>
+          <t>+921</t>
         </is>
       </c>
     </row>
@@ -33260,11 +33260,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>19340</v>
+        <v>19415</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+721</t>
+          <t>+796</t>
         </is>
       </c>
     </row>
@@ -33275,11 +33275,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>19823</v>
+        <v>19898</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+725</t>
+          <t>+800</t>
         </is>
       </c>
     </row>
@@ -33290,11 +33290,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>24038</v>
+        <v>24113</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+682</t>
+          <t>+757</t>
         </is>
       </c>
     </row>
@@ -33305,11 +33305,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>28312</v>
+        <v>28387</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+738</t>
+          <t>+813</t>
         </is>
       </c>
     </row>
@@ -33320,11 +33320,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>14965</v>
+        <v>15065</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -33410,11 +33410,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>13687</v>
+        <v>13762</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -33425,11 +33425,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>14457</v>
+        <v>14557</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -33440,11 +33440,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>14015</v>
+        <v>14115</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+871</t>
+          <t>+971</t>
         </is>
       </c>
     </row>
@@ -33455,11 +33455,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>44593</v>
+        <v>44668</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -33770,11 +33770,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>12617</v>
+        <v>12667</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1129</t>
+          <t>+1179</t>
         </is>
       </c>
     </row>
@@ -33785,11 +33785,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>12576</v>
+        <v>12626</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+1135</t>
+          <t>+1185</t>
         </is>
       </c>
     </row>
@@ -33800,11 +33800,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>12668</v>
+        <v>12718</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+1180</t>
+          <t>+1230</t>
         </is>
       </c>
     </row>
@@ -33815,11 +33815,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>7714</v>
+        <v>7739</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+1156</t>
+          <t>+1181</t>
         </is>
       </c>
     </row>
@@ -33830,11 +33830,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>7636</v>
+        <v>7661</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -34752,7 +34752,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-28 13:01:00</t>
+          <t>Timestamp: 2026-08-28 13:31:00</t>
         </is>
       </c>
     </row>
@@ -34810,11 +34810,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>27920</v>
+        <v>27945</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -34885,11 +34885,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>24801</v>
+        <v>24826</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -34900,11 +34900,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>24209</v>
+        <v>24234</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+921</t>
+          <t>+946</t>
         </is>
       </c>
     </row>
@@ -34915,11 +34915,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>24217</v>
+        <v>24242</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+942</t>
+          <t>+967</t>
         </is>
       </c>
     </row>
@@ -34930,11 +34930,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>33180</v>
+        <v>33205</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -34945,11 +34945,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>47199</v>
+        <v>47224</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+945</t>
+          <t>+970</t>
         </is>
       </c>
     </row>
@@ -35005,11 +35005,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>21417</v>
+        <v>21492</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -35020,11 +35020,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>21141</v>
+        <v>21216</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+826</t>
+          <t>+901</t>
         </is>
       </c>
     </row>
@@ -35035,11 +35035,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>21628</v>
+        <v>21703</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -35050,11 +35050,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>25814</v>
+        <v>25889</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -35065,11 +35065,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>30112</v>
+        <v>30187</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+925</t>
         </is>
       </c>
     </row>
@@ -35080,11 +35080,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>16970</v>
+        <v>16990</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1080</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -35170,11 +35170,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>15654</v>
+        <v>15679</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+992</t>
+          <t>+1017</t>
         </is>
       </c>
     </row>
@@ -35185,11 +35185,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>16549</v>
+        <v>16574</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1042</t>
+          <t>+1067</t>
         </is>
       </c>
     </row>
@@ -35200,11 +35200,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>16079</v>
+        <v>16104</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1038</t>
+          <t>+1063</t>
         </is>
       </c>
     </row>
@@ -35215,11 +35215,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>46511</v>
+        <v>46536</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1025</t>
         </is>
       </c>
     </row>
@@ -35530,11 +35530,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>14967</v>
+        <v>14992</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1128</t>
+          <t>+1153</t>
         </is>
       </c>
     </row>
@@ -35545,11 +35545,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>14926</v>
+        <v>14951</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -35560,11 +35560,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>15002</v>
+        <v>15027</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+1163</t>
+          <t>+1188</t>
         </is>
       </c>
     </row>
@@ -35575,11 +35575,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>10003</v>
+        <v>10028</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+1163</t>
+          <t>+1188</t>
         </is>
       </c>
     </row>
@@ -35590,11 +35590,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>9929</v>
+        <v>9962</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1183</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-30 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -53,6 +53,7 @@
     <sheet name="2026-08-27" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="2026-08-28" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="2026-08-29" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="2026-08-30" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36487,6 +36488,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-30 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>38489</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+4997</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Exe™</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Aline</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>8370</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>19636</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+19126</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Aline</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>8979</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>30563</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1883</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>34458</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+23539</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>21582</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+2860</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>16483</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+4912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>13232</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1718</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Lambada</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>27542</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>27575</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1986</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>26933</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1928</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>30202</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+5214</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>59037</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+25086</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>72960</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+24986</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8710</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+668</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>43125</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+16937</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>15300</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1763</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Emily Chan™</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>5016</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>30771</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+8483</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>32804</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+10788</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>28582</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+6108</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>27899</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1235</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>32256</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1303</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>32823</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+15008</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>17558</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+603</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>17498</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+594</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>17280</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+595</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>17529</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+607</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>20319</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+19052</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>23575</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+7100</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>19369</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1995</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>18881</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1977</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>55195</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+7892</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2297</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+716</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+532</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8504</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+462</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>29709</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+607</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>39173</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-9441</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>26862</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-21752</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>24580</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1094</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>21761</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-26853</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>^^Radahn</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>16268</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>25913</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+16820</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>55180</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+6566</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>4895</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>8253</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>17108</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+956</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>17013</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+937</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>17116</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+964</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>12136</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+991</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>12043</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-01 13:01:02
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -55,6 +55,7 @@
     <sheet name="2026-08-29" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-08-30" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-08-31" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="2026-09-01" sheetId="49" state="visible" r:id="rId49"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38247,6 +38248,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-01 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>38489</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Exe™</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Aline</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>8370</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>-609</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>19636</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Aline</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>8979</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>30563</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>34458</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>21582</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>16483</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>13232</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Lambada</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>27542</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>27575</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>26933</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>30202</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>59037</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>72960</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8710</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+206</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>43125</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>15300</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Emily Chan™</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>5016</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>30771</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>32804</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>28582</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>27899</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>32256</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>32823</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>17558</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>17498</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>17280</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>17529</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>20319</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>23575</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>19369</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>18881</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>55195</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2297</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8504</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>29709</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>39173</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-16007</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>26862</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-28318</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>24580</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>21761</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-33419</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>^^Radahn</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>16268</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>25913</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>55180</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>La Rata Suicida</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>4895</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>8253</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>17108</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>17013</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>17116</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>12136</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>12043</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-03 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -40911,7 +40911,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-03 13:01:00</t>
+          <t>Timestamp: 2026-09-03 13:31:00</t>
         </is>
       </c>
     </row>
@@ -41089,7 +41089,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>289</v>
+        <v>339</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -41104,7 +41104,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -41119,7 +41119,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -41134,7 +41134,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>222</v>
+        <v>272</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
@@ -41359,11 +41359,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1655</v>
+        <v>1705</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1204</t>
+          <t>+1254</t>
         </is>
       </c>
     </row>
@@ -41449,11 +41449,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>1344</v>
+        <v>1394</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1134</t>
+          <t>+1184</t>
         </is>
       </c>
     </row>
@@ -41464,11 +41464,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>1418</v>
+        <v>1443</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+1218</t>
+          <t>+1243</t>
         </is>
       </c>
     </row>
@@ -41479,11 +41479,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>1311</v>
+        <v>1336</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1206</t>
+          <t>+1231</t>
         </is>
       </c>
     </row>
@@ -41494,11 +41494,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>954</v>
+        <v>979</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+909</t>
+          <t>+934</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -41761,7 +41761,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-04 13:01:00</t>
+          <t>Timestamp: 2026-09-04 13:31:00</t>
         </is>
       </c>
     </row>
@@ -41864,11 +41864,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1872</v>
+        <v>1917</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+761</t>
+          <t>+806</t>
         </is>
       </c>
     </row>
@@ -41879,11 +41879,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1896</v>
+        <v>1941</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+721</t>
+          <t>+766</t>
         </is>
       </c>
     </row>
@@ -41894,11 +41894,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1953</v>
+        <v>2003</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+742</t>
+          <t>+792</t>
         </is>
       </c>
     </row>
@@ -41909,11 +41909,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>1907</v>
+        <v>1957</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+756</t>
+          <t>+806</t>
         </is>
       </c>
     </row>
@@ -41924,11 +41924,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>1553</v>
+        <v>1578</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1133</t>
+          <t>+1158</t>
         </is>
       </c>
     </row>
@@ -41939,11 +41939,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>1503</v>
+        <v>1516</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1118</t>
+          <t>+1131</t>
         </is>
       </c>
     </row>
@@ -41954,11 +41954,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1392</v>
+        <v>1417</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1053</t>
+          <t>+1078</t>
         </is>
       </c>
     </row>
@@ -41969,11 +41969,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>1427</v>
+        <v>1452</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1112</t>
+          <t>+1137</t>
         </is>
       </c>
     </row>
@@ -41984,11 +41984,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>1365</v>
+        <v>1390</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1075</t>
         </is>
       </c>
     </row>
@@ -41999,11 +41999,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1291</v>
+        <v>1341</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1019</t>
+          <t>+1069</t>
         </is>
       </c>
     </row>
@@ -42119,11 +42119,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2073</v>
+        <v>2098</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+829</t>
+          <t>+854</t>
         </is>
       </c>
     </row>
@@ -42149,11 +42149,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>896</v>
+        <v>951</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+388</t>
+          <t>+443</t>
         </is>
       </c>
     </row>
@@ -42164,11 +42164,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>794</v>
+        <v>838</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+313</t>
+          <t>+357</t>
         </is>
       </c>
     </row>
@@ -42179,11 +42179,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>894</v>
+        <v>926</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+415</t>
+          <t>+447</t>
         </is>
       </c>
     </row>
@@ -42194,11 +42194,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>844</v>
+        <v>904</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+396</t>
+          <t>+456</t>
         </is>
       </c>
     </row>
@@ -42209,11 +42209,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>916</v>
+        <v>976</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+410</t>
+          <t>+470</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -43491,7 +43491,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-06 13:01:00</t>
+          <t>Timestamp: 2026-09-06 13:31:00</t>
         </is>
       </c>
     </row>
@@ -43534,11 +43534,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3116</v>
+        <v>3186</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1842</t>
+          <t>+1912</t>
         </is>
       </c>
     </row>
@@ -43579,11 +43579,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>4339</v>
+        <v>4409</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+1625</t>
+          <t>+1695</t>
         </is>
       </c>
     </row>
@@ -43594,11 +43594,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>4510</v>
+        <v>4580</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1607</t>
+          <t>+1677</t>
         </is>
       </c>
     </row>
@@ -43609,11 +43609,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>4444</v>
+        <v>4514</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1514</t>
+          <t>+1584</t>
         </is>
       </c>
     </row>
@@ -43624,11 +43624,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>4323</v>
+        <v>4393</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1380</t>
+          <t>+1450</t>
         </is>
       </c>
     </row>
@@ -43639,11 +43639,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4238</v>
+        <v>4308</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1315</t>
+          <t>+1385</t>
         </is>
       </c>
     </row>
@@ -43744,11 +43744,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>4178</v>
+        <v>4248</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1567</t>
+          <t>+1637</t>
         </is>
       </c>
     </row>
@@ -43759,11 +43759,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>4132</v>
+        <v>4202</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1446</t>
+          <t>+1516</t>
         </is>
       </c>
     </row>
@@ -43774,11 +43774,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>4198</v>
+        <v>4268</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1440</t>
+          <t>+1510</t>
         </is>
       </c>
     </row>
@@ -43789,11 +43789,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>4100</v>
+        <v>4170</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1377</t>
+          <t>+1447</t>
         </is>
       </c>
     </row>
@@ -43804,11 +43804,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3978</v>
+        <v>4048</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1388</t>
+          <t>+1458</t>
         </is>
       </c>
     </row>
@@ -43834,11 +43834,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>4213</v>
+        <v>4333</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1444</t>
+          <t>+1564</t>
         </is>
       </c>
     </row>
@@ -43849,11 +43849,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>4176</v>
+        <v>4246</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1197</t>
+          <t>+1267</t>
         </is>
       </c>
     </row>
@@ -43879,11 +43879,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>3611</v>
+        <v>3681</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1705</t>
+          <t>+1775</t>
         </is>
       </c>
     </row>
@@ -43894,11 +43894,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>3486</v>
+        <v>3556</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+1709</t>
+          <t>+1779</t>
         </is>
       </c>
     </row>
@@ -43909,11 +43909,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>3485</v>
+        <v>3555</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1673</t>
+          <t>+1743</t>
         </is>
       </c>
     </row>
@@ -43924,11 +43924,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>3398</v>
+        <v>3468</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1688</t>
+          <t>+1758</t>
         </is>
       </c>
     </row>
@@ -43939,11 +43939,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>3370</v>
+        <v>3440</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1689</t>
+          <t>+1759</t>
         </is>
       </c>
     </row>
@@ -43969,11 +43969,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>2747</v>
+        <v>2817</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1583</t>
+          <t>+1653</t>
         </is>
       </c>
     </row>
@@ -44164,11 +44164,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>4307</v>
+        <v>4377</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+1886</t>
+          <t>+1956</t>
         </is>
       </c>
     </row>
@@ -44179,11 +44179,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>4171</v>
+        <v>4241</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+1750</t>
+          <t>+1820</t>
         </is>
       </c>
     </row>
@@ -44194,11 +44194,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>3814</v>
+        <v>3884</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+1471</t>
+          <t>+1541</t>
         </is>
       </c>
     </row>
@@ -44209,11 +44209,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>3963</v>
+        <v>4063</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+1542</t>
+          <t>+1642</t>
         </is>
       </c>
     </row>
@@ -44224,11 +44224,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>934</v>
+        <v>1034</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+192</t>
+          <t>+292</t>
         </is>
       </c>
     </row>
@@ -44269,11 +44269,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>873</v>
+        <v>973</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+160</t>
+          <t>+260</t>
         </is>
       </c>
     </row>
@@ -44284,11 +44284,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>3882</v>
+        <v>3982</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+1461</t>
+          <t>+1561</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-07 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -44356,7 +44356,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-07 13:01:00</t>
+          <t>Timestamp: 2026-09-07 13:31:00</t>
         </is>
       </c>
     </row>
@@ -44459,11 +44459,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>6110</v>
+        <v>6131</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1530</t>
+          <t>+1551</t>
         </is>
       </c>
     </row>
@@ -44474,11 +44474,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>6038</v>
+        <v>6063</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1524</t>
+          <t>+1549</t>
         </is>
       </c>
     </row>
@@ -44489,11 +44489,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>5893</v>
+        <v>5918</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1500</t>
+          <t>+1525</t>
         </is>
       </c>
     </row>
@@ -44504,11 +44504,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5705</v>
+        <v>5718</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1397</t>
+          <t>+1410</t>
         </is>
       </c>
     </row>
@@ -44519,11 +44519,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5977</v>
+        <v>6002</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1967</t>
+          <t>+1992</t>
         </is>
       </c>
     </row>
@@ -44534,11 +44534,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>6092</v>
+        <v>6117</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+2215</t>
+          <t>+2240</t>
         </is>
       </c>
     </row>
@@ -44549,11 +44549,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>5938</v>
+        <v>5946</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2227</t>
+          <t>+2235</t>
         </is>
       </c>
     </row>
@@ -44714,11 +44714,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>5692</v>
+        <v>5717</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1446</t>
+          <t>+1471</t>
         </is>
       </c>
     </row>
@@ -44819,11 +44819,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>6169</v>
+        <v>6194</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1547</t>
+          <t>+1572</t>
         </is>
       </c>
     </row>
@@ -44909,11 +44909,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>5353</v>
+        <v>5378</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+1326</t>
+          <t>+1351</t>
         </is>
       </c>
     </row>
@@ -44924,11 +44924,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>5744</v>
+        <v>5769</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1508</t>
+          <t>+1533</t>
         </is>
       </c>
     </row>
@@ -44939,11 +44939,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>5444</v>
+        <v>5469</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1436</t>
+          <t>+1461</t>
         </is>
       </c>
     </row>
@@ -44954,11 +44954,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>4405</v>
+        <v>4422</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1204</t>
+          <t>+1221</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-08 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -45221,7 +45221,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-08 13:01:00</t>
+          <t>Timestamp: 2026-09-08 13:31:00</t>
         </is>
       </c>
     </row>
@@ -45279,11 +45279,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>559</v>
+        <v>617</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+15</t>
+          <t>+73</t>
         </is>
       </c>
     </row>
@@ -45309,11 +45309,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>5159</v>
+        <v>5184</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+175</t>
         </is>
       </c>
     </row>
@@ -45384,11 +45384,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>6969</v>
+        <v>6994</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+967</t>
+          <t>+992</t>
         </is>
       </c>
     </row>
@@ -45399,11 +45399,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>7088</v>
+        <v>7113</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+971</t>
+          <t>+996</t>
         </is>
       </c>
     </row>
@@ -45414,11 +45414,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>6842</v>
+        <v>6867</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+896</t>
+          <t>+921</t>
         </is>
       </c>
     </row>
@@ -45429,11 +45429,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>6823</v>
+        <v>6848</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+956</t>
+          <t>+981</t>
         </is>
       </c>
     </row>
@@ -45444,11 +45444,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>6551</v>
+        <v>6572</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+972</t>
+          <t>+993</t>
         </is>
       </c>
     </row>
@@ -45459,11 +45459,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>6178</v>
+        <v>6203</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1025</t>
         </is>
       </c>
     </row>
@@ -45474,11 +45474,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>4998</v>
+        <v>5023</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+175</t>
         </is>
       </c>
     </row>
@@ -45489,11 +45489,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>4952</v>
+        <v>4960</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+158</t>
         </is>
       </c>
     </row>
@@ -45594,11 +45594,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>514</v>
+        <v>577</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+63</t>
         </is>
       </c>
     </row>
@@ -45699,11 +45699,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3934</v>
+        <v>3976</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+326</t>
+          <t>+368</t>
         </is>
       </c>
     </row>
@@ -45714,11 +45714,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>3844</v>
+        <v>3890</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+334</t>
+          <t>+380</t>
         </is>
       </c>
     </row>
@@ -45729,11 +45729,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>3687</v>
+        <v>3712</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+303</t>
+          <t>+328</t>
         </is>
       </c>
     </row>
@@ -45744,11 +45744,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>3581</v>
+        <v>3606</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+355</t>
+          <t>+380</t>
         </is>
       </c>
     </row>
@@ -45879,11 +45879,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>3405</v>
+        <v>3430</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+375</t>
+          <t>+400</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-09 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -46071,7 +46071,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-09 13:01:00</t>
+          <t>Timestamp: 2026-09-09 13:31:00</t>
         </is>
       </c>
     </row>
@@ -46159,11 +46159,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6034</v>
+        <v>6059</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -46174,11 +46174,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8002</v>
+        <v>8019</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+867</t>
         </is>
       </c>
     </row>
@@ -46189,11 +46189,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7910</v>
+        <v>7935</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -46204,11 +46204,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>7753</v>
+        <v>7778</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+855</t>
         </is>
       </c>
     </row>
@@ -46219,11 +46219,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7464</v>
+        <v>7489</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+781</t>
+          <t>+806</t>
         </is>
       </c>
     </row>
@@ -46234,11 +46234,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7824</v>
+        <v>7874</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+880</t>
         </is>
       </c>
     </row>
@@ -46249,11 +46249,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>7963</v>
+        <v>7988</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -46264,11 +46264,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>7674</v>
+        <v>7699</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+807</t>
+          <t>+832</t>
         </is>
       </c>
     </row>
@@ -46279,11 +46279,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>7711</v>
+        <v>7736</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+863</t>
+          <t>+888</t>
         </is>
       </c>
     </row>
@@ -46294,11 +46294,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>7447</v>
+        <v>7472</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+875</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -46309,11 +46309,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>7078</v>
+        <v>7103</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+875</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -46324,11 +46324,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>5845</v>
+        <v>5870</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+822</t>
+          <t>+847</t>
         </is>
       </c>
     </row>
@@ -46339,11 +46339,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>5783</v>
+        <v>5808</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+823</t>
+          <t>+848</t>
         </is>
       </c>
     </row>
@@ -46354,11 +46354,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>5893</v>
+        <v>5918</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+875</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -46369,11 +46369,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>5779</v>
+        <v>5804</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+867</t>
+          <t>+892</t>
         </is>
       </c>
     </row>
@@ -46384,11 +46384,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>5649</v>
+        <v>5665</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+851</t>
+          <t>+867</t>
         </is>
       </c>
     </row>
@@ -46429,11 +46429,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>7538</v>
+        <v>7563</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+821</t>
+          <t>+846</t>
         </is>
       </c>
     </row>
@@ -46549,11 +46549,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>4497</v>
+        <v>4522</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+521</t>
+          <t>+546</t>
         </is>
       </c>
     </row>
@@ -46729,11 +46729,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>3880</v>
+        <v>3930</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+500</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -46921,7 +46921,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-10 13:01:00</t>
+          <t>Timestamp: 2026-09-10 13:31:00</t>
         </is>
       </c>
     </row>
@@ -47024,11 +47024,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8778</v>
+        <v>8803</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+759</t>
+          <t>+784</t>
         </is>
       </c>
     </row>
@@ -47039,11 +47039,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>8718</v>
+        <v>8743</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+783</t>
+          <t>+808</t>
         </is>
       </c>
     </row>
@@ -47054,11 +47054,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>8570</v>
+        <v>8595</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+792</t>
+          <t>+817</t>
         </is>
       </c>
     </row>
@@ -47069,11 +47069,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>8277</v>
+        <v>8302</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+788</t>
+          <t>+813</t>
         </is>
       </c>
     </row>
@@ -47084,11 +47084,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>8939</v>
+        <v>9009</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1065</t>
+          <t>+1135</t>
         </is>
       </c>
     </row>
@@ -47099,11 +47099,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>9067</v>
+        <v>9142</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1079</t>
+          <t>+1154</t>
         </is>
       </c>
     </row>
@@ -47114,11 +47114,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>8753</v>
+        <v>8828</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1054</t>
+          <t>+1129</t>
         </is>
       </c>
     </row>
@@ -47129,11 +47129,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>8844</v>
+        <v>8919</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1108</t>
+          <t>+1183</t>
         </is>
       </c>
     </row>
@@ -47144,11 +47144,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>8569</v>
+        <v>8644</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1097</t>
+          <t>+1172</t>
         </is>
       </c>
     </row>
@@ -47159,11 +47159,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>8192</v>
+        <v>8242</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1089</t>
+          <t>+1139</t>
         </is>
       </c>
     </row>
@@ -47279,11 +47279,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>8363</v>
+        <v>8388</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+825</t>
         </is>
       </c>
     </row>
@@ -47399,11 +47399,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>5293</v>
+        <v>5318</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+771</t>
+          <t>+796</t>
         </is>
       </c>
     </row>
@@ -47414,11 +47414,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>5090</v>
+        <v>5115</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+772</t>
+          <t>+797</t>
         </is>
       </c>
     </row>
@@ -47429,11 +47429,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>4971</v>
+        <v>4996</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+825</t>
         </is>
       </c>
     </row>
@@ -47444,11 +47444,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>4829</v>
+        <v>4854</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+792</t>
+          <t>+817</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-11 13:31:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -47771,7 +47771,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-11 13:01:00</t>
+          <t>Timestamp: 2026-09-11 13:31:00</t>
         </is>
       </c>
     </row>
@@ -47934,11 +47934,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>10099</v>
+        <v>10149</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1090</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -47949,11 +47949,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>10238</v>
+        <v>10288</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1096</t>
+          <t>+1146</t>
         </is>
       </c>
     </row>
@@ -47964,11 +47964,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>9896</v>
+        <v>9946</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1068</t>
+          <t>+1118</t>
         </is>
       </c>
     </row>
@@ -47979,11 +47979,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>9991</v>
+        <v>10041</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1072</t>
+          <t>+1122</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-13 13:01:01
</commit_message>
<xml_diff>
--- a/clan_3094.xlsx
+++ b/clan_3094.xlsx
@@ -67,6 +67,7 @@
     <sheet name="2026-09-10" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="2026-09-11" sheetId="59" state="visible" r:id="rId59"/>
     <sheet name="2026-09-12" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="2026-09-13" sheetId="61" state="visible" r:id="rId61"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50295,6 +50296,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Sangre Latina Clan (3094)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-13 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>8020</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1591</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Kyara Senju™</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>5975</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+510</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Exe™</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3182</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Ereshkigal</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>7920</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+510</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Killua Senju™</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>10271</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Tsunade Senju™</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10308</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mito Senju™</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>10152</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Hisoka Senju™</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>9862</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Lambada</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>11288</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Orpheus</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>11451</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Ahrtheus</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>11177</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Euridice</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>11176</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Atenea</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>11014</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Persefone</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>10533</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>ll</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7812</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>lll</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7786</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+623</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>IV</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>7810</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7548</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+441</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7419</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1579</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>-121</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Himawari</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>8650</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1332</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Chrollo Senju™</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>9929</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+123</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Emily Chan™</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3201</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+641</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drako </t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>6565</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+473</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Azusa Chan</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>6397</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Arceus</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>6315</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+464</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fenraim </t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>6277</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Thurzin</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>6277</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tamara Anbu</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>10302</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Yügao | Anbu</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>8074</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1687</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Hinoko | Anbu</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>7897</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1705</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Kunoichi | Anbu</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7777</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1687</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Kaguya | Anbu</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>7536</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1646</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Sabrina Carpenter</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1563</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Haku Anbu</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>9333</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Arch"</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>9867</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Kushina</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>9466</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Lucia</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>8117</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Rosangel</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2039</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Wisin y Yandel</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Taylor Swift</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Rö | Anbu</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>7379</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1655</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>6383</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1086</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>6941</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1644</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>....</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>5794</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>6098</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+801</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>^^Radahn</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>3462</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+491</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Zheninjas</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Jounin Gakure</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Bicho</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>3166</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>_ D E X T E R _</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>5997</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>ShaToshi</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>1742</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>